<commit_message>
docs: test case csv and update in xlsx
</commit_message>
<xml_diff>
--- a/Test_Cases/23127052_Test_Cases.xlsx
+++ b/Test_Cases/23127052_Test_Cases.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DaiHoc\KiemThuPM\HW06\Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A26B16CC-D68F-4B4F-AD8D-E977338ACAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FFB00FE-FECC-4200-A755-84B7B6865870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8A65A0A-E0D1-48B6-95FB-FFF48A20EC99}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C8A65A0A-E0D1-48B6-95FB-FFF48A20EC99}"/>
   </bookViews>
   <sheets>
     <sheet name="23127052_FR04_Test_Cases" sheetId="1" r:id="rId1"/>
     <sheet name="23127052_FR07_Test_Cases" sheetId="2" r:id="rId2"/>
+    <sheet name="23127052_FR14_Test_Cases" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="407">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -870,6 +871,378 @@
   </si>
   <si>
     <t>TC_FR07_01</t>
+  </si>
+  <si>
+    <t>TC_FR14_01</t>
+  </si>
+  <si>
+    <t>FR-14: Quản lý Danh mục (Category CRUD)</t>
+  </si>
+  <si>
+    <t>POST /api/categories</t>
+  </si>
+  <si>
+    <t>[Schema] Response đúng định dạng JSON Object</t>
+  </si>
+  <si>
+    <t>Kiểm tra phản hồi trả về từ API phải là một JSON Object hợp lệ khi tạo thành công (HTTP 200/201).</t>
+  </si>
+  <si>
+    <t>200 OK / 201 Created</t>
+  </si>
+  <si>
+    <t>TC_FR14_02</t>
+  </si>
+  <si>
+    <t>[Schema] Response chứa đúng các trường bắt buộc ('message', 'id')</t>
+  </si>
+  <si>
+    <t>Kiểm tra response có thuộc tính message ('Category created') và id kiểu số nguyên dương.</t>
+  </si>
+  <si>
+    <t>TC_FR14_03</t>
+  </si>
+  <si>
+    <t>[Schema] Response không chứa các trường thừa không xác định</t>
+  </si>
+  <si>
+    <t>Kiểm tra response chỉ chứa chính xác 2 trường message và id, không rò rỉ dữ liệu nội bộ.</t>
+  </si>
+  <si>
+    <t>TC_FR14_04</t>
+  </si>
+  <si>
+    <t>[Schema] Validate toàn bộ response với JSON Schema (tv4/ajv)</t>
+  </si>
+  <si>
+    <t>Dùng thư viện schema validation của Postman để đối chiếu cấu trúc JSON response 100%.</t>
+  </si>
+  <si>
+    <t>TC_FR14_05</t>
+  </si>
+  <si>
+    <t>[Domain - Valid] Tạo danh mục với tên tiếng Việt có dấu</t>
+  </si>
+  <si>
+    <t>Body {"name": "Đồng hồ thông minh"} -&gt; Kỳ vọng HTTP 200/201 OK.</t>
+  </si>
+  <si>
+    <t>TC_FR14_06</t>
+  </si>
+  <si>
+    <t>[Domain - Valid] Tạo danh mục với tên tiếng Anh không dấu</t>
+  </si>
+  <si>
+    <t>Body {"name": "Smart Watch"} -&gt; Kỳ vọng HTTP 200/201 OK.</t>
+  </si>
+  <si>
+    <t>TC_FR14_07</t>
+  </si>
+  <si>
+    <t>[Domain - Valid] Tạo danh mục với tên chứa chữ số</t>
+  </si>
+  <si>
+    <t>Body {"name": "iPhone 15 Series"} -&gt; Kỳ vọng HTTP 200/201 OK.</t>
+  </si>
+  <si>
+    <t>TC_FR14_08</t>
+  </si>
+  <si>
+    <t>[Domain - Valid] Tên chứa ký tự đặc biệt thông dụng (&amp;, -, /)</t>
+  </si>
+  <si>
+    <t>Body {"name": "Âm thanh &amp; Phụ kiện"} -&gt; Kỳ vọng HTTP 200/201 OK.</t>
+  </si>
+  <si>
+    <t>TC_FR14_09</t>
+  </si>
+  <si>
+    <t>[Domain - Valid] Tên đạt độ dài tối thiểu (1 ký tự)</t>
+  </si>
+  <si>
+    <t>Body {"name": "A"} -&gt; Kỳ vọng HTTP 200/201 OK.</t>
+  </si>
+  <si>
+    <t>TC_FR14_10</t>
+  </si>
+  <si>
+    <t>[Domain - Valid] Tên đạt độ dài tối đa hợp lệ (255 ký tự)</t>
+  </si>
+  <si>
+    <t>Body {"name": "a".repeat(255)} -&gt; Kỳ vọng HTTP 200/201 OK.</t>
+  </si>
+  <si>
+    <t>TC_FR14_11</t>
+  </si>
+  <si>
+    <t>[Domain - Valid] Tên chứa khoảng trắng ở đầu và cuối</t>
+  </si>
+  <si>
+    <t>Body {"name": "  Máy tính bảng  "} -&gt; Kỳ vọng HTTP 200/201 OK, hệ thống tự động trim.</t>
+  </si>
+  <si>
+    <t>TC_FR14_12</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Tên danh mục là chuỗi rỗng ('')</t>
+  </si>
+  <si>
+    <t>Body {"name": ""} -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_13</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Tên danh mục chỉ chứa toàn khoảng trắng ('   ')</t>
+  </si>
+  <si>
+    <t>Body {"name": "   "} -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_14</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Thiếu trường name trong request body</t>
+  </si>
+  <si>
+    <t>Body {} -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_15</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Trường name có giá trị null</t>
+  </si>
+  <si>
+    <t>Body {"name": null} -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_16</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Trường name có kiểu dữ liệu số nguyên (12345)</t>
+  </si>
+  <si>
+    <t>Body {"name": 12345} -&gt; Xử lý an toàn (HTTP 400 hoặc ép kiểu chuỗi).</t>
+  </si>
+  <si>
+    <t>TC_FR14_17</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Trường name có kiểu dữ liệu boolean (true)</t>
+  </si>
+  <si>
+    <t>Body {"name": true} -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_18</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Trường name có kiểu dữ liệu mảng ([])</t>
+  </si>
+  <si>
+    <t>Body {"name": ["Thời trang"]} -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_19</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Trường name có kiểu dữ liệu object ({})</t>
+  </si>
+  <si>
+    <t>Body {"name": {"sub": "con"}} -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_20</t>
+  </si>
+  <si>
+    <t>[Domain - Invalid] Tên danh mục vượt quá độ dài tối đa (256 ký tự)</t>
+  </si>
+  <si>
+    <t>Body {"name": "a".repeat(256)} -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_21</t>
+  </si>
+  <si>
+    <t>[Domain - Edge] Request body hoàn toàn rỗng (Empty payload)</t>
+  </si>
+  <si>
+    <t>Raw body "" -&gt; Kỳ vọng HTTP 400 Bad Request.</t>
+  </si>
+  <si>
+    <t>TC_FR14_22</t>
+  </si>
+  <si>
+    <t>[Domain - Edge] Gửi kèm trường không xác định ngoài name</t>
+  </si>
+  <si>
+    <t>Body {"name": "Gia dụng", "extra_field": "test"} -&gt; Xử lý an toàn (bỏ qua hoặc 400).</t>
+  </si>
+  <si>
+    <t>TC_FR14_23</t>
+  </si>
+  <si>
+    <t>[State] POST response trả về id mới hợp lệ (&gt; 0)</t>
+  </si>
+  <si>
+    <t>Xác nhận id trả về là số nguyên dương và lưu vào biến môi trường latest_created_category_id.</t>
+  </si>
+  <si>
+    <t>TC_FR14_24</t>
+  </si>
+  <si>
+    <t>[State - Chained] Gọi GET /api/categories trả về HTTP 200 OK</t>
+  </si>
+  <si>
+    <t>Gửi request GET /api/categories qua pm.sendRequest để đọc danh sách danh mục hiện tại.</t>
+  </si>
+  <si>
+    <t>TC_FR14_25</t>
+  </si>
+  <si>
+    <t>[State - Chained] Danh mục vừa tạo xuất hiện trong GET /api/categories</t>
+  </si>
+  <si>
+    <t>Tìm kiếm trong mảng danh mục có phần tử thỏa mãn item.id === createdId.</t>
+  </si>
+  <si>
+    <t>TC_FR14_26</t>
+  </si>
+  <si>
+    <t>[State - Chained] Tên danh mục trong CSDL khớp với name đã gửi</t>
+  </si>
+  <si>
+    <t>Đối chiếu foundCategory.name trả về từ GET với reqBody.name gửi lên trong POST.</t>
+  </si>
+  <si>
+    <t>TC_FR14_27</t>
+  </si>
+  <si>
+    <t>[State - Chained] Mọi danh mục trong danh sách đều có cấu trúc {id, name}</t>
+  </si>
+  <si>
+    <t>Duyệt qua mảng kết quả của GET và kiểm tra từng item đều có đầy đủ id và name.</t>
+  </si>
+  <si>
+    <t>TC_FR14_28</t>
+  </si>
+  <si>
+    <t>[State] Xử lý khi tạo danh mục trùng tên đã tồn tại</t>
+  </si>
+  <si>
+    <t>Gửi tên trùng với danh mục đã có trong hệ thống -&gt; Kiểm tra phản hồi (200/201/409).</t>
+  </si>
+  <si>
+    <t>200 OK / 409 Conflict</t>
+  </si>
+  <si>
+    <t>TC_FR14_29</t>
+  </si>
+  <si>
+    <t>[Security - SEC-02] Không gửi Authorization Header -&gt; Bị từ chối 401</t>
+  </si>
+  <si>
+    <t>Gửi request không có token -&gt; Kỳ vọng HTTP 401 Unauthorized.</t>
+  </si>
+  <si>
+    <t>TC_FR14_30</t>
+  </si>
+  <si>
+    <t>[Security - SEC-02] Gửi Token không hợp lệ hoặc hết hạn -&gt; Bị từ chối 401</t>
+  </si>
+  <si>
+    <t>Gửi Authorization: Bearer INVALID_TOKEN -&gt; Kỳ vọng HTTP 401 Unauthorized.</t>
+  </si>
+  <si>
+    <t>TC_FR14_31</t>
+  </si>
+  <si>
+    <t>[Security - SEC-03] Kiểm tra phân quyền Admin: User thường không được tạo danh mục</t>
+  </si>
+  <si>
+    <t>FR-12: Chỉ role Admin mới được tạo danh mục. Dùng token user thường (test@eshop.com) -&gt; Kỳ vọng HTTP 403.</t>
+  </si>
+  <si>
+    <t>403 Forbidden</t>
+  </si>
+  <si>
+    <t>TC_FR14_32</t>
+  </si>
+  <si>
+    <t>[Security - SEC-05 / SQLi] Tấn công SQL Injection vào trường name</t>
+  </si>
+  <si>
+    <t>Payload {"name": "' OR 1=1 --"} hoặc DROP TABLE -&gt; Kỳ vọng không sập 500 DB.</t>
+  </si>
+  <si>
+    <t>TC_FR14_33</t>
+  </si>
+  <si>
+    <t>[Security - SEC-04 / XSS] Tấn công Stored XSS vào trường name</t>
+  </si>
+  <si>
+    <t>Payload {"name": "&lt;script&gt;alert('XSS')&lt;/script&gt;"} -&gt; Không crash 500, sanitize an toàn khi đọc lại.</t>
+  </si>
+  <si>
+    <t>TC_FR14_34</t>
+  </si>
+  <si>
+    <t>[Security - IDOR / Tampering] Client tự ý chỉ định trường id trong body</t>
+  </si>
+  <si>
+    <t>Body {"name": "Test", "id": 9999} -&gt; Server tự sinh ID, không cho phép ghi đè ID theo ý client.</t>
+  </si>
+  <si>
+    <t>TC_FR14_35</t>
+  </si>
+  <si>
+    <t>[Security - Content-Type] Gửi payload dạng XML / Text thay vì JSON</t>
+  </si>
+  <si>
+    <t>Đặt header Content-Type: application/xml -&gt; Kỳ vọng HTTP 400 hoặc 415 Unsupported Media Type.</t>
+  </si>
+  <si>
+    <t>TC_FR14_E1</t>
+  </si>
+  <si>
+    <t>[Security] Gửi payload tên danh mục cực lớn (DoS)</t>
+  </si>
+  <si>
+    <t>Truyền chuỗi name vài Megabytes -&gt; Expect HTTP 413 Payload Too Large.</t>
+  </si>
+  <si>
+    <t>TC_FR14_E2</t>
+  </si>
+  <si>
+    <t>Gửi request bằng method PUT hoặc PATCH tới /api/categories thay vì POST -&gt; Expect HTTP 405 Method Not Allowed.</t>
+  </si>
+  <si>
+    <t>TC_FR14_E3</t>
+  </si>
+  <si>
+    <t>[Security / Race Condition] Tạo đồng thời danh mục trùng tên</t>
+  </si>
+  <si>
+    <t>Bắn 2 request POST /api/categories cùng tên trong khoảng 10ms -&gt; Expect xử lý tuần tự, không tạo 2 danh mục trùng lặp rác.</t>
+  </si>
+  <si>
+    <t>TC_FR14_E4</t>
+  </si>
+  <si>
+    <t>[Format] Tên chứa ký tự khoảng trắng tàng hình (Zero-width space)</t>
+  </si>
+  <si>
+    <t>Truyền tên danh mục chứa ký tự xuống dòng (\n) hoặc Zero-width space (\u200B) -&gt; Expect HTTP 400 hoặc làm sạch an toàn.</t>
+  </si>
+  <si>
+    <t>TC_FR14_E5</t>
+  </si>
+  <si>
+    <t>[State] Kiểm tra trạng thái mặc định của danh mục mới</t>
+  </si>
+  <si>
+    <t>Sau khi POST thành công, gọi GET /api/categories kiểm tra danh mục mới được tự động kích hoạt hiển thị (is_active: true).</t>
   </si>
 </sst>
 </file>
@@ -1766,7 +2139,7 @@
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="19.5703125" customWidth="1"/>
     <col min="4" max="4" width="18.85546875" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
     <col min="6" max="6" width="44.140625" customWidth="1"/>
     <col min="7" max="7" width="83" customWidth="1"/>
     <col min="8" max="8" width="42.42578125" customWidth="1"/>
@@ -3034,7 +3407,7 @@
     <col min="2" max="2" width="30.85546875" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="19.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" customWidth="1"/>
     <col min="6" max="6" width="54.5703125" customWidth="1"/>
     <col min="7" max="7" width="103" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
@@ -4233,4 +4606,1214 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A274766-E597-4B39-831A-8D881C653627}">
+  <dimension ref="A1:I41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" customWidth="1"/>
+    <col min="6" max="6" width="69.42578125" customWidth="1"/>
+    <col min="7" max="7" width="100.7109375" customWidth="1"/>
+    <col min="8" max="8" width="39.140625" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>